<commit_message>
updated parse_floorplan and pdf_parser files
</commit_message>
<xml_diff>
--- a/boq_styled.xlsx
+++ b/boq_styled.xlsx
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -686,32 +686,62 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>SUPERSTRUCTURE WORKS</t>
-        </is>
-      </c>
       <c r="B2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Superstructure Works</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
         <v>123400</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>FINISHES</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Finishes</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
         <v>4202920</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B10" s="8" t="n">
         <v>4326320</v>
       </c>
     </row>

</xml_diff>